<commit_message>
Docs: Yiwei MG04254FRA1S1N / MG0425-UB-60-4P as alternates to Adafruit #5358 / #5412 (J3 order unchanged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Claude outputs/AI_Calculator_Shopping_List.xlsx
+++ b/Claude outputs/AI_Calculator_Shopping_List.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="P31" s="17" t="inlineStr">
         <is>
-          <t>Legs straightened into J3. Meter-check against the cable before gluing.</t>
+          <t>Legs straightened into J3. Meter-check against the cable before gluing. Alternate (2026-10-10, from Nirav): Yiwei MG04254FRA1S1N is the same part as #5358. Not price-checked.</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="P32" s="17" t="inlineStr">
         <is>
-          <t>Charges AND flashes. Stock was ~35 on 10/6: order first. Backup: Jameco / DigiKey.</t>
+          <t>Charges AND flashes. Stock was ~35 on 10/6: order first. Backup: Jameco / DigiKey. Alternate (2026-10-10, from Nirav): Yiwei MG0425-UB-60-4P = equivalent of #5412; reads GND, D+, D−, V+ from its N end, like #5412. Same J3 order (1 VBUS, 2 D−, 3 D+, 4 GND, N end at pin 1) and the same meter check before gluing. Not price-checked.</t>
         </is>
       </c>
     </row>

</xml_diff>